<commit_message>
site - 22.07 plan
</commit_message>
<xml_diff>
--- a/Grafik_CCEE_SLIVEN1_19_07_2026.xlsx
+++ b/Grafik_CCEE_SLIVEN1_19_07_2026.xlsx
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="B10" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="B11" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
@@ -813,7 +813,7 @@
         </is>
       </c>
       <c r="B12" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="B13" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
@@ -857,7 +857,7 @@
         </is>
       </c>
       <c r="B14" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B15" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="B16" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
@@ -923,7 +923,7 @@
         </is>
       </c>
       <c r="B17" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="B18" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="B19" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="B20" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
@@ -1011,7 +1011,7 @@
         </is>
       </c>
       <c r="B21" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="B22" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
@@ -1055,7 +1055,7 @@
         </is>
       </c>
       <c r="B23" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="B24" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
@@ -1099,7 +1099,7 @@
         </is>
       </c>
       <c r="B25" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="B26" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="B27" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
@@ -1165,7 +1165,7 @@
         </is>
       </c>
       <c r="B28" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="B29" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
@@ -1209,7 +1209,7 @@
         </is>
       </c>
       <c r="B30" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="B31" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
@@ -1253,7 +1253,7 @@
         </is>
       </c>
       <c r="B32" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="B33" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
@@ -1297,7 +1297,7 @@
         </is>
       </c>
       <c r="B34" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="B35" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="B36" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
@@ -1363,7 +1363,7 @@
         </is>
       </c>
       <c r="B37" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
@@ -1385,7 +1385,7 @@
         </is>
       </c>
       <c r="B38" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
@@ -1407,7 +1407,7 @@
         </is>
       </c>
       <c r="B39" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
@@ -1429,7 +1429,7 @@
         </is>
       </c>
       <c r="B40" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C40" s="10" t="inlineStr">
         <is>
@@ -1451,7 +1451,7 @@
         </is>
       </c>
       <c r="B41" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
         </is>
       </c>
       <c r="B42" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C42" s="10" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="B43" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="B44" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C44" s="10" t="inlineStr">
         <is>
@@ -1539,7 +1539,7 @@
         </is>
       </c>
       <c r="B45" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="B46" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C46" s="10" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
         </is>
       </c>
       <c r="B47" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
@@ -1605,7 +1605,7 @@
         </is>
       </c>
       <c r="B48" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="B49" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
@@ -1649,7 +1649,7 @@
         </is>
       </c>
       <c r="B50" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="B51" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="B52" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
@@ -1715,7 +1715,7 @@
         </is>
       </c>
       <c r="B53" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="B54" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
@@ -1759,7 +1759,7 @@
         </is>
       </c>
       <c r="B55" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
@@ -1781,7 +1781,7 @@
         </is>
       </c>
       <c r="B56" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C56" s="10" t="inlineStr">
         <is>
@@ -1803,7 +1803,7 @@
         </is>
       </c>
       <c r="B57" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="B58" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
@@ -1847,12 +1847,10 @@
         </is>
       </c>
       <c r="B59" s="1" t="n">
-        <v>46222</v>
-      </c>
-      <c r="C59" s="10" t="inlineStr">
-        <is>
-          <t>Put Adex Solcast value here</t>
-        </is>
+        <v>46217</v>
+      </c>
+      <c r="C59" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="D59" s="5" t="n">
         <v>0</v>
@@ -1869,7 +1867,7 @@
         </is>
       </c>
       <c r="B60" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C60" s="11" t="n">
         <v>0</v>
@@ -1889,7 +1887,7 @@
         </is>
       </c>
       <c r="B61" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C61" s="11" t="n">
         <v>0</v>
@@ -1909,7 +1907,7 @@
         </is>
       </c>
       <c r="B62" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C62" s="11" t="n">
         <v>0</v>
@@ -1929,7 +1927,7 @@
         </is>
       </c>
       <c r="B63" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C63" s="11" t="n">
         <v>0</v>
@@ -1949,7 +1947,7 @@
         </is>
       </c>
       <c r="B64" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C64" s="11" t="n">
         <v>0</v>
@@ -1969,7 +1967,7 @@
         </is>
       </c>
       <c r="B65" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C65" s="11" t="n">
         <v>0</v>
@@ -1989,7 +1987,7 @@
         </is>
       </c>
       <c r="B66" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C66" s="11" t="n">
         <v>0</v>
@@ -2009,7 +2007,7 @@
         </is>
       </c>
       <c r="B67" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C67" s="11" t="n">
         <v>0</v>
@@ -2029,7 +2027,7 @@
         </is>
       </c>
       <c r="B68" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C68" s="11" t="n">
         <v>0</v>
@@ -2049,7 +2047,7 @@
         </is>
       </c>
       <c r="B69" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C69" s="11" t="n">
         <v>0</v>
@@ -2069,7 +2067,7 @@
         </is>
       </c>
       <c r="B70" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C70" s="11" t="n">
         <v>0</v>
@@ -2089,7 +2087,7 @@
         </is>
       </c>
       <c r="B71" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C71" s="11" t="n">
         <v>0</v>
@@ -2109,7 +2107,7 @@
         </is>
       </c>
       <c r="B72" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C72" s="11" t="n">
         <v>0</v>
@@ -2129,7 +2127,7 @@
         </is>
       </c>
       <c r="B73" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C73" s="11" t="n">
         <v>0</v>
@@ -2149,7 +2147,7 @@
         </is>
       </c>
       <c r="B74" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C74" s="11" t="n">
         <v>0</v>
@@ -2169,10 +2167,12 @@
         </is>
       </c>
       <c r="B75" s="1" t="n">
-        <v>46222</v>
-      </c>
-      <c r="C75" s="11" t="n">
-        <v>0</v>
+        <v>46217</v>
+      </c>
+      <c r="C75" s="10" t="inlineStr">
+        <is>
+          <t>Put Adex Solcast value here</t>
+        </is>
       </c>
       <c r="D75" s="5" t="n">
         <v>0</v>
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="B76" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C76" s="10" t="inlineStr">
         <is>
@@ -2211,7 +2211,7 @@
         </is>
       </c>
       <c r="B77" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C77" s="10" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="B78" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C78" s="10" t="inlineStr">
         <is>
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="B79" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C79" s="10" t="inlineStr">
         <is>
@@ -2277,7 +2277,7 @@
         </is>
       </c>
       <c r="B80" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C80" s="10" t="inlineStr">
         <is>
@@ -2299,7 +2299,7 @@
         </is>
       </c>
       <c r="B81" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C81" s="10" t="inlineStr">
         <is>
@@ -2321,7 +2321,7 @@
         </is>
       </c>
       <c r="B82" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C82" s="10" t="inlineStr">
         <is>
@@ -2343,7 +2343,7 @@
         </is>
       </c>
       <c r="B83" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C83" s="10" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="B84" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C84" s="10" t="inlineStr">
         <is>
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="B85" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C85" s="10" t="inlineStr">
         <is>
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="B86" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C86" s="10" t="inlineStr">
         <is>
@@ -2431,7 +2431,7 @@
         </is>
       </c>
       <c r="B87" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C87" s="10" t="inlineStr">
         <is>
@@ -2453,7 +2453,7 @@
         </is>
       </c>
       <c r="B88" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C88" s="10" t="inlineStr">
         <is>
@@ -2475,7 +2475,7 @@
         </is>
       </c>
       <c r="B89" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C89" s="10" t="inlineStr">
         <is>
@@ -2497,7 +2497,7 @@
         </is>
       </c>
       <c r="B90" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C90" s="10" t="inlineStr">
         <is>
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="B91" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C91" s="10" t="inlineStr">
         <is>
@@ -2541,7 +2541,7 @@
         </is>
       </c>
       <c r="B92" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C92" s="10" t="inlineStr">
         <is>
@@ -2563,7 +2563,7 @@
         </is>
       </c>
       <c r="B93" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C93" s="10" t="inlineStr">
         <is>
@@ -2585,7 +2585,7 @@
         </is>
       </c>
       <c r="B94" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C94" s="11" t="n">
         <v>0</v>
@@ -2605,7 +2605,7 @@
         </is>
       </c>
       <c r="B95" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C95" s="11" t="n">
         <v>0</v>
@@ -2625,7 +2625,7 @@
         </is>
       </c>
       <c r="B96" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C96" s="11" t="n">
         <v>0</v>
@@ -2645,7 +2645,7 @@
         </is>
       </c>
       <c r="B97" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C97" s="11" t="n">
         <v>0</v>
@@ -2665,7 +2665,7 @@
         </is>
       </c>
       <c r="B98" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C98" s="11" t="n">
         <v>0</v>
@@ -2685,7 +2685,7 @@
         </is>
       </c>
       <c r="B99" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C99" s="11" t="n">
         <v>0</v>
@@ -2705,7 +2705,7 @@
         </is>
       </c>
       <c r="B100" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C100" s="11" t="n">
         <v>0</v>
@@ -2725,7 +2725,7 @@
         </is>
       </c>
       <c r="B101" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C101" s="11" t="n">
         <v>0</v>
@@ -2745,7 +2745,7 @@
         </is>
       </c>
       <c r="B102" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C102" s="11" t="n">
         <v>0</v>
@@ -2765,7 +2765,7 @@
         </is>
       </c>
       <c r="B103" s="1" t="n">
-        <v>46222</v>
+        <v>46217</v>
       </c>
       <c r="C103" s="11" t="n">
         <v>0</v>

</xml_diff>